<commit_message>
ACDR2026: closing remarks draft; scenario updates (YI-Lab speaker, photo duty, summary by DG)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing の登壇者（Summary＝ADRC、Closing Remarks＝三浦センター長＋SCDF側）は Sylvia と要確認。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       <c r="O3" s="5" t="inlineStr">
         <is>
           <t>写真
-(藤本/塩見)</t>
+(藤本/塩見/荒木田)</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
@@ -3507,7 +3507,7 @@
       <c r="O3" s="5" t="inlineStr">
         <is>
           <t>写真
-(藤本/塩見)</t>
+(藤本/塩見/荒木田)</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
@@ -4458,14 +4458,14 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Our fourth presentation is from YI-Lab (Nepal). May I invite YI-Lab, Nepal. Please.
+          <t>Our fourth presentation is from YI-Lab (Nepal). May I invite Mr Pradip Khatiwada, YI-Lab, Nepal. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>YI-Lab, Nepal【氏名 TBC】</t>
+          <t>Mr Pradip Khatiwada, YI-Lab, Nepal</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -4840,7 +4840,7 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>所要15分。Summary（ADRC）6分＋閉会挨拶 2名×3分＋MC連絡3分。登壇者【TBC】。</t>
+          <t>所要15分。Summary（宮木所長）6分＋閉会挨拶 2名×3分（三浦センター長、SCDF代表【TBC】）＋MC連絡3分。</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -4868,24 +4868,24 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>PPT 20: Closing Title → PPT 21: ACDR2026 Summary（Gerry 作成）</t>
+          <t>PPT 20: Closing Title → PPT 21: ACDR2026 Summary（Gerry 起草・宮木所長発表）</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Ladies and gentlemen, please be seated. We now come to the summary and closing of ACDR2026. First, I invite Dr. Gerald Potutan, Deputy Director for Research of the Asian Disaster Reduction Center, to present the summary of the conference.
+          <t>Ladies and gentlemen, please be seated. We now come to the summary and closing of ACDR2026. First, I invite Mr MIYAKI Kazuhiro, Director General of the Asian Disaster Reduction Center, to present the summary of the conference.
 （Summary 約6分）
-Thank you, Dr. Potutan.</t>
+Thank you, Mr Miyaki.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>発表者は Gerry か宮木所長か【TBC】（2025年は所長がまとめ）。</t>
+          <t>Summary は Gerry が起草（28日夜〜29日朝）、宮木所長が発表（2025年と同じく所長）。</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Gerry（演台）</t>
+          <t>宮木所長（演台）</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>閉会挨拶案は Opening 案の末尾に短文を付す（別紙）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>6枠: Google / JAXA / BRIN / YI-Lab / Uzbekistan / Cabinet Office of Japan (Spectee + 1)</t>
+          <t>6枠: Google (Ms Sirada Boonkongchuen) / JAXA / BRIN (Dr Yenni Vetrita) / YI-Lab (Mr Pradip Khatiwada) / Uzbekistan / Cabinet Office of Japan (Spectee + 1)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>氏名は 10/9 確定後</t>
+          <t>未確定の氏名は 10/9 確定後</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       <c r="D19" s="7" t="inlineStr">
         <is>
           <t>ACDR2026 Summary and Closing Remarks
-– Summary: Asian Disaster Reduction Center
+– Summary: Mr MIYAKI Kazuhiro, Director General, ADRC
 – Closing Remarks: Prof. MIURA Fusanori, Chairman, ADRC / [SCDF]</t>
         </is>
       </c>
@@ -5690,7 +5690,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Gerry 作成（RT・TS の要点）</t>
+          <t>Gerry 起草・宮木所長発表（RT・TS の要点）</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: closing remarks by Executive Director Kitamoto
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝北本 Executive Director＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>所要15分。Summary（宮木所長）6分＋閉会挨拶 2名×3分（三浦センター長、SCDF代表【TBC】）＋MC連絡3分。</t>
+          <t>所要15分。Summary（宮木所長）6分＋閉会挨拶 2名×3分（北本 Executive Director、SCDF代表【TBC】）＋MC連絡3分。三浦センター長は着席。</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -4939,24 +4939,24 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>PPT 22: Name（三浦センター長）</t>
+          <t>PPT 22: Name（北本 Executive Director）</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Now I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, for his closing remarks.
+          <t>Now I would like to invite Mr KITAMOTO Masayuki, Executive Director of the Asian Disaster Reduction Center, for his closing remarks.
 （閉会挨拶 約3分）
-Thank you very much, Professor Miura.</t>
+Thank you very much, Mr Kitamoto.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_KITAMOTO_案0929.docx（約3分）。肩書 Executive Director は 11/1 付だが名簿と同じ表記を使用（荒木田 9/29）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Prof. Miura（演台）</t>
+          <t>北本 ED（演台）</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -5667,7 +5667,7 @@
         <is>
           <t>ACDR2026 Summary and Closing Remarks
 – Summary: Mr MIYAKI Kazuhiro, Director General, ADRC
-– Closing Remarks: Prof. MIURA Fusanori, Chairman, ADRC / [SCDF]</t>
+– Closing Remarks: Mr KITAMOTO Masayuki, Executive Director, ADRC / [SCDF]</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>三浦センター長 / SCDF 代表</t>
+          <t>北本 Executive Director / SCDF 代表</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: closing remarks by Executive Director Miyaki (October title); fix summary title
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝北本 Executive Director＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝宮木所長（Executive Director）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>所要15分。Summary（宮木所長）6分＋閉会挨拶 2名×3分（北本 Executive Director、SCDF代表【TBC】）＋MC連絡3分。三浦センター長は着席。</t>
+          <t>所要15分。Summary 6分＋ADRC 閉会挨拶 3分（いずれも宮木所長＝Executive Director、演台に留まる）＋SCDF 代表 3分【TBC】＋MC連絡3分。三浦センター長は着席。</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -4873,14 +4873,14 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Ladies and gentlemen, please be seated. We now come to the summary and closing of ACDR2026. First, I invite Mr MIYAKI Kazuhiro, Director General of the Asian Disaster Reduction Center, to present the summary of the conference.
+          <t>Ladies and gentlemen, please be seated. We now come to the summary and closing of ACDR2026. First, I invite Mr MIYAKI Kazuhiro, Executive Director of the Asian Disaster Reduction Center, to present the summary of the conference.
 （Summary 約6分）
 Thank you, Mr Miyaki.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Summary は Gerry が起草（28日夜〜29日朝）、宮木所長が発表（2025年と同じく所長）。</t>
+          <t>Summary は Gerry が起草（28日夜〜29日朝）、宮木所長（Executive Director、10月時点の肩書）が発表。</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -4939,24 +4939,24 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>PPT 22: Name（北本 Executive Director）</t>
+          <t>PPT 22: Name（宮木所長 Executive Director）</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Now I would like to invite Mr KITAMOTO Masayuki, Executive Director of the Asian Disaster Reduction Center, for his closing remarks.
+          <t>Thank you, Mr Miyaki. Please stay at the lectern: I now invite you, as Executive Director of the Asian Disaster Reduction Center, to deliver the closing remarks on behalf of ADRC.
 （閉会挨拶 約3分）
-Thank you very much, Mr Kitamoto.</t>
+Thank you very much, Mr Miyaki.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_KITAMOTO_案0929.docx（約3分）。肩書 Executive Director は 11/1 付だが名簿と同じ表記を使用（荒木田 9/29）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIYAKI_案0929.docx（約3分）。Summary に続けて同じ登壇者が閉会挨拶（演台に留まる）。三浦センター長は着席。次回 ACDR 開催地の発表があればここ【TBC】。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>北本 ED（演台）</t>
+          <t>宮木所長（演台・続き）</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -5666,8 +5666,8 @@
       <c r="D19" s="7" t="inlineStr">
         <is>
           <t>ACDR2026 Summary and Closing Remarks
-– Summary: Mr MIYAKI Kazuhiro, Director General, ADRC
-– Closing Remarks: Mr KITAMOTO Masayuki, Executive Director, ADRC / [SCDF]</t>
+– Summary: Mr MIYAKI Kazuhiro, Executive Director, ADRC
+– Closing Remarks: Mr MIYAKI Kazuhiro, Executive Director, ADRC / [SCDF]</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>北本 Executive Director / SCDF 代表</t>
+          <t>宮木所長 Executive Director / SCDF 代表</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: closing remarks by Chairman Miura, summary by Executive Director Miyaki
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝宮木所長（Executive Director）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>所要15分。Summary 6分＋ADRC 閉会挨拶 3分（いずれも宮木所長＝Executive Director、演台に留まる）＋SCDF 代表 3分【TBC】＋MC連絡3分。三浦センター長は着席。</t>
+          <t>所要15分。Summary（宮木所長＝Executive Director）6分＋閉会挨拶 2名×3分（三浦センター長＝Chairman、SCDF 代表【TBC】）＋MC連絡3分。</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -4939,24 +4939,24 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>PPT 22: Name（宮木所長 Executive Director）</t>
+          <t>PPT 22: Name（三浦センター長 Chairman）</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Thank you, Mr Miyaki. Please stay at the lectern: I now invite you, as Executive Director of the Asian Disaster Reduction Center, to deliver the closing remarks on behalf of ADRC.
+          <t>Now I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, for his closing remarks.
 （閉会挨拶 約3分）
-Thank you very much, Mr Miyaki.</t>
+Thank you very much, Professor Miura.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_MIYAKI_案0929.docx（約3分）。Summary に続けて同じ登壇者が閉会挨拶（演台に留まる）。三浦センター長は着席。次回 ACDR 開催地の発表があればここ【TBC】。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>宮木所長（演台・続き）</t>
+          <t>Prof. Miura（演台）</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -5667,7 +5667,7 @@
         <is>
           <t>ACDR2026 Summary and Closing Remarks
 – Summary: Mr MIYAKI Kazuhiro, Executive Director, ADRC
-– Closing Remarks: Mr MIYAKI Kazuhiro, Executive Director, ADRC / [SCDF]</t>
+– Closing Remarks: Prof. MIURA Fusanori, Chairman, ADRC / [SCDF]</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>宮木所長 Executive Director / SCDF 代表</t>
+          <t>三浦センター長（Chairman） / SCDF 代表</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: announce next ACDR in Sendai in closing remarks
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR 開催地の発表があればここ【TBC】。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催（挨拶内で発表、時期は要確認）。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: next ACDR back to back with APMCDRR in Sendai
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催、APMCDRR と back-to-back（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催（挨拶内で発表、時期は要確認）。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催、APMCDRR と back-to-back（挨拶内で発表、時期は要確認）。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: next ACDR in Sendai, October 2027
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -548,7 +548,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催、APMCDRR と back-to-back（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
+          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催、APMCDRR と back-to-back、2027年10月（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催、APMCDRR と back-to-back（挨拶内で発表、時期は要確認）。</t>
+          <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催、APMCDRR と back-to-back、2027年10月（挨拶内で発表）。</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026 scenario: evaluation form by ADRC; interpretation for Deputy Minister to be confirmed with CAO
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B14"/>
+  <dimension ref="B1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="2" max="2"/>
@@ -566,6 +566,13 @@
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>未確定は【TBC】で示す。人名は 0925 参加者名簿の綴りに合わせた。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>未確定事項の確認先: 内閣府＝林副大臣の使用言語・通訳方式。ADRC＝評価フォーム（用意・URL/QR）、RT の質問方式、Co-Moderator の要否。Sylvia（SCDF/COSEM）＝Commissioner の出席、Closing の SCDF 登壇者、フィールドトリップ集合場所、会場バナー前の写真。</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1093,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>逐次通訳を入れると所要が倍になる。日本語で話す場合は英訳原稿を事前配布し通訳は要点のみ、または英語原稿の読み上げを内閣府（足立氏）と要調整【TBC】。挨拶後、林副大臣は Japan 席に着席、その後退席（Japan 席は内閣府参事官に交代）。</t>
+          <t>逐次通訳を入れると所要が倍になる。日本語で話す場合は英訳原稿を事前配布し通訳は要点のみ、または英語原稿の読み上げ。使用言語・通訳の方式は内閣府に確認【TBC・ADRC→内閣府】。挨拶後、林副大臣は Japan 席に着席、その後退席（Japan 席は内閣府参事官に交代）。</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -5084,7 +5091,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>評価フォーム URL/QR【TBC】。フィールドトリップ集合場所【TBC】（田中: 名簿・点呼）。パレード前のホテル着替え・再移動は最終案内に記載。</t>
+          <t>評価フォームは ADRC が用意（Google Form 等、URL/QR を PPT 24 に。担当【TBC】）。フィールドトリップ集合場所【TBC】（田中: 名簿・点呼）。パレード前のホテル着替え・再移動は最終案内に記載。</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -5750,7 +5757,7 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>URL TBC</t>
+          <t>ADRC が用意（2023 は bit.ly 短縮 URL＋QR）。URL 確定後に差替</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ACDR2026 RT: alphabetical order, 5 min per member country, adviser/ADPC/orgs after; mail draft updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -527,14 +527,14 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>・時間配分の仮定: 開会挨拶 各4分（3名＋MCで15分）。RT ステートメントは各国4分（2023年タジキスタンと同じ、ベル方式）、日本・仙台市は5分（9/25内閣府連絡会）、国際機関・オブザーバーは3分。TS は rev1.0（紹介5分＋発表15分×6枠＋質疑15分＋まとめ10分）。</t>
+          <t>・時間配分: 開会挨拶 各4分（3名＋MCで15分）。RT はメンバー国 各5分まで（荒木田 9/29 決定、ベル方式）、アドバイザー国・ADPC・その他機関は3分（仮）。TS は rev1.0（紹介5分＋発表15分×6枠＋質疑15分＋まとめ10分）。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>・RT 発言順は「主催側（Singapore→Japan→仙台市）→メンバー国アルファベット順→国際機関」の案。登録国（9/16版10か国＋追加）で当日までに確定し、未登録国の行は削除する。</t>
+          <t>・RT 発言順（荒木田 9/29 決定）: メンバー国アルファベット順（Japan の直後に仙台市）→ 希望があればアドバイザー国（AUS/NZ）→ ADPC → その他機関アルファベット順（ADB, AHA Centre, Google, オンライン UNDP/WMO）。Part 1 は Armenia〜Turkiye（22枠×5分＝13:03〜14:53）、Part 2 は Uzbekistan・Viet Nam＋機関。登録国で当日までに確定し、未登録国の行は削除する。</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P43"/>
+  <dimension ref="B1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1313,7 +1313,7 @@
       <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Excellencies, distinguished delegates. The Roundtable is the session where ADRC member countries and partners share, in their own words, the progress they have made under the Sendai Framework for Disaster Risk Reduction and the challenges that remain as we approach 2030. Part 1 is held this afternoon and Part 2 tomorrow morning at 9 o’clock.
-Each delegation is invited to make a statement of up to four minutes; the Government of Japan and the City of Sendai have five minutes; partner organisations have three minutes. Please speak from your seat using the table microphone. A bell will ring once when one minute remains, twice at thirty seconds, and three times at the end of your time. To keep the programme on schedule, I ask all speakers to observe the time strictly.
+Member countries are invited to make a statement of up to five minutes, in alphabetical order; adviser countries and partner organisations will follow with up to three minutes each. Please speak from your seat using the table microphone. A bell will ring once when one minute remains, twice at thirty seconds, and three times at the end of your time. To keep the programme on schedule, I ask all speakers to observe the time strictly.
 Questions and comments will not be taken on the floor during the statements; please write them on the comment sheet at your seat [or submit them via the online form shown on the screen]. They will be shared with the speakers and reflected in the conference summary.</t>
         </is>
       </c>
@@ -1364,29 +1364,29 @@
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Singapore</t>
+          <t>Statement: the delegation of Armenia</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-1: Singapore</t>
+          <t>PPT 09-1: Armenia</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Singapore, Singapore Civil Defence Force. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Armenia. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>主催側として最初に発言。Commissioner か Alan Chow 氏か【TBC】。</t>
+          <t>アルメニアとアゼルバイジャンは配席上離してあるが、発言順はアルファベット順で連続（荒木田 9/29 決定）。</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -1439,629 +1439,629 @@
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>13:09</t>
+          <t>13:08</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
+          <t>Statement: the delegation of Azerbaijan</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-2: Azerbaijan</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Azerbaijan. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of Bangladesh</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-3: Bangladesh</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Bangladesh. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of Bhutan</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-4: Bhutan</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Bhutan. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of Brunei Darussalam</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-5: Brunei Darussalam</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Brunei Darussalam. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of Cambodia</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-6: Cambodia</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Cambodia. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of Fiji</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-7: Fiji</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of Fiji. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Statement: the delegation of India</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-8: India</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite the delegation of India. You have 5 minutes, please.
+（ステートメント 5分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>着席発言（卓上マイク）</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>国名スライド</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>卓上マイク ON 確認</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Q&amp;A欄監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
           <t>Statement: the delegation of Japan</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-2: Japan</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-9: Japan</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Japan, Cabinet Office. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>林副大臣は Opening 後に退席予定のため、日本のステートメントは内閣府参事官【TBC】。</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>13:14</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Statement: Mr TAKAHASHI Shinichi</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-3: City of Sendai</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>PPT 09-10: City of Sendai</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite Mr TAKAHASHI Shinichi, Vice Mayor of the City of Sendai, Japan. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>教室列1列目の卓上マイクから発言（配席表0928）。次期 APMCDRR ホスト市としての紹介を含む見込み。</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P18" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>13:19</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Armenia</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-4: Armenia</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Armenia. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>アルメニアとアゼルバイジャンは配席上離してある。発言順もアルファベット順で連続するが、間に挟む国を置くかは要判断【TBC】。</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L19" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P19" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>13:23</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Azerbaijan</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-5: Azerbaijan</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Azerbaijan. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P20" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>13:27</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Bangladesh</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-6: Bangladesh</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Bangladesh. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P21" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>13:31</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Bhutan</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-7: Bhutan</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Bhutan. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O22" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P22" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>13:35</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Brunei Darussalam</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-8: Brunei Darussalam</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Brunei Darussalam. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P23" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>13:39</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Cambodia</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-9: Cambodia</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Cambodia. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
-        </is>
-      </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>着席発言（卓上マイク）</t>
-        </is>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>国名スライド</t>
-        </is>
-      </c>
-      <c r="K24" s="7" t="inlineStr">
-        <is>
-          <t>卓上マイク ON 確認</t>
-        </is>
-      </c>
-      <c r="L24" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者</t>
-        </is>
-      </c>
-      <c r="M24" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N24" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O24" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P24" s="7" t="inlineStr">
-        <is>
-          <t>Q&amp;A欄監視</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>13:43</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Statement: the delegation of Fiji</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>PPT 09-10: Fiji</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite the delegation of Fiji. You have 4 minutes, please.
-（ステートメント 4分）
-Thank you very much.</t>
-        </is>
-      </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+          <t>日本の直後に仙台市（教室列1列目の卓上マイク）。次期 APMCDRR・ACDR2027 ホスト市としての紹介を含む見込み。</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -2114,23 +2114,23 @@
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:53</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of India</t>
+          <t>Statement: the delegation of Lao PDR</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-11: India</t>
+          <t>PPT 09-11: Lao PDR</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of India. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Lao PDR. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2189,23 +2189,23 @@
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Lao PDR</t>
+          <t>Statement: the delegation of Malaysia</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-12: Lao PDR</t>
+          <t>PPT 09-12: Malaysia</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Lao PDR. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Malaysia. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2264,23 +2264,23 @@
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Malaysia</t>
+          <t>Statement: the delegation of Maldives</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-13: Malaysia</t>
+          <t>PPT 09-13: Maldives</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Malaysia. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Maldives. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2339,23 +2339,23 @@
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Maldives</t>
+          <t>Statement: the delegation of Mongolia</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-14: Maldives</t>
+          <t>PPT 09-14: Mongolia</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Maldives. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Mongolia. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2414,23 +2414,23 @@
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Mongolia</t>
+          <t>Statement: the delegation of Myanmar</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-15: Mongolia</t>
+          <t>PPT 09-15: Myanmar</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Mongolia. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Myanmar. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2489,23 +2489,23 @@
       <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Myanmar</t>
+          <t>Statement: the delegation of Pakistan</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-16: Myanmar</t>
+          <t>PPT 09-16: Pakistan</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Myanmar. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Pakistan. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2564,23 +2564,23 @@
       <c r="B32" s="7" t="n"/>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Pakistan</t>
+          <t>Statement: the delegation of Papua New Guinea</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-17: Pakistan</t>
+          <t>PPT 09-17: Papua New Guinea</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Pakistan. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Papua New Guinea. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2639,23 +2639,23 @@
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Papua New Guinea</t>
+          <t>Statement: the delegation of Republic of Korea</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-18: Papua New Guinea</t>
+          <t>PPT 09-18: Republic of Korea</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Papua New Guinea. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Republic of Korea. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
@@ -2714,29 +2714,29 @@
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Republic of Korea</t>
+          <t>Statement: the delegation of Singapore</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-19: Republic of Korea</t>
+          <t>PPT 09-19: Singapore</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Republic of Korea. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Singapore. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
+          <t>アルファベット順どおり Singapore の位置。Commissioner か Alan Chow 氏か【TBC】。</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -2789,34 +2789,34 @@
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Statement: the Asian Disaster Preparedness Center</t>
+          <t>Statement: the delegation of Sri Lanka</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>PPT 10-1: ADPC</t>
+          <t>PPT 09-20: Sri Lanka</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the Asian Disaster Preparedness Center, ADPC. You have three minutes, please.
-（ステートメント 3分）
+          <t>Next, I would like to invite the delegation of Sri Lanka. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>ADPC は Observer 組織。教室列1列目から発言。</t>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>着席発言</t>
+          <t>着席発言（卓上マイク）</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -2826,17 +2826,17 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>組織スライド</t>
+          <t>国名スライド</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>マイク</t>
+          <t>卓上マイク ON 確認</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者／Zoom</t>
+          <t>カメラ: 発言者</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>オンライン登壇者のスポットライト</t>
+          <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
@@ -2864,34 +2864,34 @@
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Statement: the AHA Centre</t>
+          <t>Statement: the delegation of Thailand</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>PPT 10-2: AHA Centre</t>
+          <t>PPT 09-21: Thailand</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the AHA Centre. You have three minutes, please.
-（ステートメント 3分）
+          <t>Next, I would like to invite the delegation of Thailand. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>RT 発言の可能性大（9/29）。卓上マイクなし→スタンド/ハンドマイク。</t>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>着席発言</t>
+          <t>着席発言（卓上マイク）</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
@@ -2901,17 +2901,17 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>組織スライド</t>
+          <t>国名スライド</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>マイク</t>
+          <t>卓上マイク ON 確認</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者／Zoom</t>
+          <t>カメラ: 発言者</t>
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>オンライン登壇者のスポットライト</t>
+          <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
@@ -2939,34 +2939,34 @@
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Statement: the Asian Development Bank</t>
+          <t>Statement: the delegation of Turkiye</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>PPT 10-3: ADB</t>
+          <t>PPT 09-22: Turkiye</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the Asian Development Bank, ADB. You have three minutes, please.
-（ステートメント 3分）
+          <t>Next, I would like to invite the delegation of Turkiye. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>発言は未定（9/29 JM6）。</t>
+          <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>着席発言</t>
+          <t>着席発言（卓上マイク）</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -2976,17 +2976,17 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>組織スライド</t>
+          <t>国名スライド</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>マイク</t>
+          <t>卓上マイク ON 確認</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者／Zoom</t>
+          <t>カメラ: 発言者</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>オンライン登壇者のスポットライト</t>
+          <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
@@ -3014,56 +3014,50 @@
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:53</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Statement: the National Emergency Management Agency of New Zealand</t>
+          <t>予備時間・Part 1 締め</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>PPT 10-4: New Zealand</t>
+          <t>PPT 11: Comments &amp; Questions（提出方法）</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the National Emergency Management Agency of New Zealand. You have three minutes, please.
-（ステートメント 3分）
-Thank you very much.</t>
+          <t>We have a few minutes before the end of Part 1. If any delegation wishes to add a brief comment on what we have heard, please raise your name plate. [If none:] Please also use the comment sheets on your desk; they will be collected by the secretariat during the coffee break.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>アドバイザー国。SIDEX 側プログラムとの兼ね合いで出席者【TBC】。</t>
+          <t>進行が押した場合はこの枠を吸収に使う。</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>着席発言</t>
+          <t>Moderator</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>紹介・御礼</t>
+          <t>進行</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>組織スライド</t>
+          <t>PPT 11</t>
         </is>
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>マイク</t>
-        </is>
-      </c>
-      <c r="L38" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者／Zoom</t>
-        </is>
-      </c>
+          <t>スタンド/ハンドマイク</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="n"/>
       <c r="M38" s="7" t="inlineStr">
         <is>
           <t>記録</t>
@@ -3074,324 +3068,105 @@
           <t>記録</t>
         </is>
       </c>
-      <c r="O38" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P38" s="7" t="inlineStr">
-        <is>
-          <t>オンライン登壇者のスポットライト</t>
-        </is>
-      </c>
+      <c r="O38" s="7" t="n"/>
+      <c r="P38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Statement: Google</t>
+          <t>RT Part 1 まとめ・連絡事項</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>PPT 10-5: Google</t>
+          <t>PPT 12: Info（Coffee / SC / Gala）</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite Google. You have three minutes, please.
-（ステートメント 3分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>教室列1列目の卓上マイクから発言。</t>
-        </is>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>着席発言</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>組織スライド</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>マイク</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者／Zoom</t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N39" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr">
-        <is>
-          <t>オンライン登壇者のスポットライト</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>14:38</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>Statement: online participants [UNDP / WMO]</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>PPT 10-6: Online</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Next, I would like to invite online participants [UNDP / WMO]. You have three minutes, please.
-（ステートメント 3分）
-Thank you very much.</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>オンライン登壇は未登録。Zoom 側の映像・音声を会場スクリーンへ（藤本・神戸）。</t>
-        </is>
-      </c>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>着席発言</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>紹介・御礼</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>組織スライド</t>
-        </is>
-      </c>
-      <c r="K40" s="7" t="inlineStr">
-        <is>
-          <t>マイク</t>
-        </is>
-      </c>
-      <c r="L40" s="7" t="inlineStr">
-        <is>
-          <t>カメラ: 発言者／Zoom</t>
-        </is>
-      </c>
-      <c r="M40" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N40" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O40" s="7" t="inlineStr">
-        <is>
-          <t>発言者写真</t>
-        </is>
-      </c>
-      <c r="P40" s="7" t="inlineStr">
-        <is>
-          <t>オンライン登壇者のスポットライト</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>14:41</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>Open floor / comments（予備時間）</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>PPT 11: Comments &amp; Questions（提出方法）</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>We have a few minutes before the end of Part 1. If any delegation wishes to add a brief comment on what we have heard, please raise your name plate. [If none:] Please also use the comment sheets on your desk; they will be collected by the secretariat during the coffee break.</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>進行が押した場合はこの枠を吸収に使う。</t>
-        </is>
-      </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>Moderator</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="inlineStr">
-        <is>
-          <t>進行</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>PPT 11</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="inlineStr">
-        <is>
-          <t>スタンド/ハンドマイク</t>
-        </is>
-      </c>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N41" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="7" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>14:55</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>RT Part 1 まとめ・連絡事項</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>PPT 12: Info（Coffee / SC / Gala）</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>Thank you to all the delegations for your statements. This concludes Part 1 of the Roundtable. The remaining statements will be heard tomorrow morning in Part 2, starting at 9 o’clock sharp in this room.
 Three announcements. First, coffee is served in front of this room. Second, the Steering Committee Meeting for ADRC member countries only will start at 15:15 in this room. Delegates of member countries, please return by 15:15. Third, for participants attending the SIDEX Gala Dinner, the bus leaves Dorsett Changi City Hotel at 17:30. Thank you.</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>SC の前方席: 議長＝内閣府参事官、ADRC（所長）。SC 開始までに机上の RT 資料を回収（吉田・塩見）。</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>Moderator</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>読み上げ</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>PPT 12</t>
         </is>
       </c>
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="K39" s="7" t="n"/>
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>Webinar 一時停止（SC は別 Zoom）</t>
         </is>
       </c>
-      <c r="M42" s="7" t="inlineStr">
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="N42" s="7" t="inlineStr">
+      <c r="N39" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="O42" s="7" t="n"/>
-      <c r="P42" s="7" t="inlineStr">
+      <c r="O39" s="7" t="n"/>
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>録画停止・保存</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="6" t="n">
+    <row r="40">
+      <c r="B40" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>15:00-15:15</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Coffee Break</t>
         </is>
       </c>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>コーヒー: Peridot 前。SC 用に前方席の名札を差し替え（吉田・田中）。Gerry は RT ノートを整理し Summary 執筆へ。</t>
         </is>
       </c>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
-      <c r="M43" s="6" t="n"/>
-      <c r="N43" s="6" t="n"/>
-      <c r="O43" s="6" t="n"/>
-      <c r="P43" s="6" t="n"/>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="6" t="n"/>
+      <c r="L40" s="6" t="n"/>
+      <c r="M40" s="6" t="n"/>
+      <c r="N40" s="6" t="n"/>
+      <c r="O40" s="6" t="n"/>
+      <c r="P40" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3404,7 +3179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P30"/>
+  <dimension ref="B1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3631,7 +3406,7 @@
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>残り5か国（Sri Lanka, Thailand, Turkiye, Uzbekistan, Viet Nam）＋まとめ。各4分。</t>
+          <t>残り2か国（Uzbekistan, Viet Nam、各5分）→ アドバイザー国（希望があれば）→ ADPC → その他機関アルファベット順（ADB, AHA Centre, Google, オンライン）各3分 → まとめ。全員が発言すると約5分超過。未登録分が緩衝。</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -3664,7 +3439,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Good morning, Excellencies, distinguished delegates. Welcome back to the Roundtable Session, Part 2. We will hear the remaining statements, again with four minutes each and the same bell signals as yesterday.</t>
+          <t>Good morning, Excellencies, distinguished delegates. Welcome back to the Roundtable Session, Part 2. We will hear the remaining member-country statements, again with five minutes each, followed by statements from adviser countries and partner organisations with three minutes each. The bell signals are the same as yesterday.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -3711,22 +3486,26 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Sri Lanka</t>
+          <t>Statement: the delegation of Uzbekistan</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-20: Sri Lanka</t>
+          <t>PPT 09-23: Uzbekistan</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Sri Lanka. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Uzbekistan. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G8" s="7" t="n"/>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>登録確認【TBC】</t>
+        </is>
+      </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
@@ -3777,31 +3556,27 @@
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Thailand</t>
+          <t>Statement: the delegation of Viet Nam</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-21: Thailand</t>
+          <t>PPT 09-24: Viet Nam</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Thailand. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the delegation of Viet Nam. You have 5 minutes, please.
+（ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>登録確認【TBC】</t>
-        </is>
-      </c>
+      <c r="G9" s="7" t="n"/>
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
@@ -3852,30 +3627,34 @@
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Turkiye</t>
+          <t>Statement: the National Emergency Management Agency of New Zealand</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-22: Turkiye</t>
+          <t>PPT 10-1: New Zealand</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Turkiye. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the National Emergency Management Agency of New Zealand. You have three minutes, please.
+（ステートメント 3分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G10" s="7" t="n"/>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>アドバイザー国（希望があれば）。AUS NEMA も出席・希望があればここ。</t>
+        </is>
+      </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>着席発言（卓上マイク）</t>
+          <t>着席発言</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -3885,17 +3664,17 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>国名スライド</t>
+          <t>組織スライド</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>卓上マイク ON 確認</t>
+          <t>マイク</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者</t>
+          <t>カメラ: 発言者／Zoom</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -3915,7 +3694,7 @@
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>Q&amp;A欄監視</t>
+          <t>オンライン登壇者のスポットライト</t>
         </is>
       </c>
     </row>
@@ -3923,34 +3702,34 @@
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Uzbekistan</t>
+          <t>Statement: the Asian Disaster Preparedness Center</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-23: Uzbekistan</t>
+          <t>PPT 10-2: ADPC</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Uzbekistan. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the Asian Disaster Preparedness Center, ADPC. You have three minutes, please.
+（ステートメント 3分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>登録確認【TBC】</t>
+          <t>Observer 組織。アドバイザー国の次。</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>着席発言（卓上マイク）</t>
+          <t>着席発言</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -3960,17 +3739,17 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>国名スライド</t>
+          <t>組織スライド</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>卓上マイク ON 確認</t>
+          <t>マイク</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者</t>
+          <t>カメラ: 発言者／Zoom</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -3990,7 +3769,7 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Q&amp;A欄監視</t>
+          <t>オンライン登壇者のスポットライト</t>
         </is>
       </c>
     </row>
@@ -4003,25 +3782,29 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Statement: the delegation of Viet Nam</t>
+          <t>Statement: the Asian Development Bank</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>PPT 09-24: Viet Nam</t>
+          <t>PPT 10-3: ADB</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Viet Nam. You have 4 minutes, please.
-（ステートメント 4分）
+          <t>Next, I would like to invite the Asian Development Bank, ADB. You have three minutes, please.
+（ステートメント 3分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>その他機関はアルファベット順。発言は未定（9/29 JM6）。</t>
+        </is>
+      </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>着席発言（卓上マイク）</t>
+          <t>着席発言</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -4031,17 +3814,17 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>国名スライド</t>
+          <t>組織スライド</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>卓上マイク ON 確認</t>
+          <t>マイク</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>カメラ: 発言者</t>
+          <t>カメラ: 発言者／Zoom</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
@@ -4061,7 +3844,7 @@
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>Q&amp;A欄監視</t>
+          <t>オンライン登壇者のスポットライト</t>
         </is>
       </c>
     </row>
@@ -4069,47 +3852,56 @@
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>RT まとめ</t>
+          <t>Statement: the AHA Centre</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>PPT 11: Comments &amp; Questions</t>
+          <t>PPT 10-4: AHA Centre</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Thank you very much to all the delegations. Over the two parts of this Roundtable we have heard from [23] member countries and [6] partner organisations. The key points will be reflected in the conference summary presented at the closing at 11:45. Comment sheets can still be handed to the secretariat until the coffee break.
-We will now move to the Technical Session. Speakers of the Technical Session, please take your seats at the front.</t>
+          <t>Next, I would like to invite the AHA Centre. You have three minutes, please.
+（ステートメント 3分）
+Thank you very much.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Gerry がここまでの内容を Summary に反映（執筆時間: 28日夜〜29日朝）。前方席への登壇者移動（池田誘導）。</t>
+          <t>RT 発言の可能性大（9/29）。卓上マイクなし→スタンド/ハンドマイク。</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Moderator</t>
+          <t>着席発言</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>進行</t>
+          <t>紹介・御礼</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>PPT 11</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
+          <t>組織スライド</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>マイク</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者／Zoom</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>記録</t>
@@ -4120,1048 +3912,1264 @@
           <t>記録</t>
         </is>
       </c>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>オンライン登壇者のスポットライト</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Technical Session: DRR DX for Isolated and Inaccessible Regions: Redefining Community Resilience through Advanced Technologies</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Moderator: LTC Chen Yong Kai（SCDF）。Co-Chair: Dr. Mizan Bisri（ADRC/ADPC）。PIC: 池田。AV/Zoom: 荒木田。カメラ・フロア: 塩見。配分（rev1.0）: 紹介5分＋発表15分×6＋質疑15分＋まとめ10分。</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="6" t="n"/>
-      <c r="P14" s="6" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Statement: Google</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>PPT 10-5: Google</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite Google. You have three minutes, please.
+（ステートメント 3分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>教室列1列目の卓上マイクから発言。</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>着席発言</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>組織スライド</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>マイク</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者／Zoom</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>オンライン登壇者のスポットライト</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Statement: online participants [UNDP / WMO]</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>PPT 10-6: Online</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Next, I would like to invite online participants [UNDP / WMO]. You have three minutes, please.
+（ステートメント 3分）
+Thank you very much.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>オンライン登壇は未登録。Zoom 側の映像・音声を会場スクリーンへ（藤本・神戸）。</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>着席発言</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>紹介・御礼</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>組織スライド</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>マイク</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>カメラ: 発言者／Zoom</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>発言者写真</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>オンライン登壇者のスポットライト</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>RT まとめ</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>PPT 11: Comments &amp; Questions</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Thank you very much to all the delegations. Over the two parts of this Roundtable we have heard from [23] member countries, [adviser countries] and [5] partner organisations. The key points will be reflected in the conference summary presented at the closing at 11:45. Comment sheets can still be handed to the secretariat until the coffee break.
+We will now move to the Technical Session. Speakers of the Technical Session, please take your seats at the front.</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Gerry がここまでの内容を Summary に反映（執筆時間: 28日夜〜29日朝）。前方席への登壇者移動（池田誘導）。</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Moderator</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>進行</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>PPT 11</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Technical Session: DRR DX for Isolated and Inaccessible Regions: Redefining Community Resilience through Advanced Technologies</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Moderator: LTC Chen Yong Kai（SCDF）。Co-Chair: Dr. Mizan Bisri（ADRC/ADPC）。PIC: 池田。AV/Zoom: 荒木田。カメラ・フロア: 塩見。配分（rev1.0）: 紹介5分＋発表15分×6＋質疑15分＋まとめ10分。</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>TS 趣旨・登壇者紹介</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>PPT 14: TS Title（Moderator / Co-Chair）→ PPT 15: Speakers（6枠・組織名と氏名）→ PPT 16: Instruction for Presenters（15分、ベル）</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Ladies and gentlemen, we now begin the Technical Session on “DRR DX for Isolated and Inaccessible Regions: Redefining Community Resilience through Advanced Technologies”. I am joined by our Co-Chair, Dr. Mizan Bisri of the Asian Disaster Reduction Center.
 [Co-Chair, 2 minutes: session objective — how advanced technologies (satellite EO, AI, communications) can keep isolated communities informed and connected before, during and after disasters; link to the Roundtable and to the ADRC concept note.]
 We have six presentations of fifteen minutes each, followed by fifteen minutes of questions and answers and a wrap-up. Presenters, please speak from the lectern. A bell will ring at one minute remaining, at thirty seconds, and at the end. Questions will be taken together after all presentations; please note your questions and the presenter’s name.</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>コンセプトノート rev1.2（Central Asia and Caucasus 表記）。PPT 15 の氏名は 10/9 確定後に入れる（対外資料は組織名のみ）。</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Moderator / Co-Chair（モデレーター卓）</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>進行</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>PPT 14→16</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>モデレーター卓マイク</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台固定＋会場</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>09:35</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Presentation 1: Google</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>PPT 17-1: Name（Google）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Our first presentation is from Google. May I invite Ms Sirada Boonkongchuen, Product Partnership, Google Search &amp; Gemini, Google. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Ms Sirada Boonkongchuen, Product Partnership, Google Search &amp; Gemini, Google</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N16" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P16" s="7" t="inlineStr">
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>09:50</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Presentation 2: JAXA</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>PPT 17-2: Name（JAXA）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Our second presentation is from JAXA. May I invite Japan Aerospace Exploration Agency (JAXA). Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>Japan Aerospace Exploration Agency (JAXA)【発表者 2名から選定中】</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L20" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P20" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>10:05</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Presentation 3: BRIN</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>PPT 17-3: Name（BRIN）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Our third presentation is from BRIN. May I invite Dr. Yenni Vetrita, Researcher, Research Center for Geoinformatics, National Research and Innovation Agency (BRIN), Indonesia. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Dr. Yenni Vetrita, Researcher, Research Center for Geoinformatics, National Research and Innovation Agency (BRIN), Indonesia</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L21" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P18" s="7" t="inlineStr">
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>10:20</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Presentation 4: YI-Lab (Nepal)</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>PPT 17-4: Name（YI-Lab (Nepal)）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Our fourth presentation is from YI-Lab (Nepal). May I invite Mr Pradip Khatiwada, YI-Lab, Nepal. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>Mr Pradip Khatiwada, YI-Lab, Nepal</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L22" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr">
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P19" s="7" t="inlineStr">
+      <c r="P22" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Presentation 5: Uzbekistan</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>PPT 17-5: Name（Uzbekistan）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Our fifth presentation is from Uzbekistan. May I invite Uzbekistan (ADRC member country). Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Uzbekistan (ADRC member country)【回答待ち】</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="L23" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr">
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P20" s="7" t="inlineStr">
+      <c r="P23" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>10:50</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Presentation 6: Japan (Cabinet Office)</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>PPT 17-6: Name（Japan (Cabinet Office)）→ 発表スライド</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Our sixth presentation is from Japan (Cabinet Office). May I invite Cabinet Office, Government of Japan: 1-minute introduction + Spectee + one more company. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Cabinet Office, Government of Japan: 1-minute introduction + Spectee + one more company【TBC】（計15分）
 内閣府枠は中根氏が1分イントロ。前方席8席の入替なし。</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>演台（クリッカー1本）</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>スライド切替</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P21" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>11:05</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>PPT 18: Q&amp;A</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>We now have fifteen minutes for questions. Please raise your hand or your name plate, state your name and organisation, and address your question to a specific presenter. We will take two or three questions at a time. [Co-Chair reads selected online questions.]</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>スタンド/ハンドマイクを塩見が回す。オンライン質問は神戸（中村）→ 藤本 → Co-Chair。</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Moderator / Co-Chair</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>進行</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>PPT 18</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>ハンドマイク2</t>
         </is>
       </c>
-      <c r="L22" s="7" t="inlineStr">
+      <c r="L25" s="7" t="inlineStr">
         <is>
           <t>Zoom Q&amp;A 取次</t>
         </is>
       </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="inlineStr">
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="n"/>
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A 取次</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>11:20</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>TS まとめ</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>PPT 19: Wrap-up</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>[Co-Chair, 8 minutes: three to four take-aways across the six presentations; how they answer the session question; items for the conference summary.]
-[Moderator:] Thank you, Dr. Mizan, and thank you to all six presenters. This concludes the Technical Session. Coffee is served in front of the room; please be back by 11:45 for the summary and closing.</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>TS 要旨は原稿ベースで事前に概要案（池田・Mizan→Gerry）。</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Co-Chair → Moderator</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>御礼・連絡</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>PPT 19</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>11:30-11:45</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Coffee Break</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Gerry: Summary スライド最終化（RT Part 2・TS を反映）。前方登壇者席の名札を撤去、閉会用に三浦センター長・SCDF代表の席札。</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
-      <c r="M24" s="6" t="n"/>
-      <c r="N24" s="6" t="n"/>
-      <c r="O24" s="6" t="n"/>
-      <c r="P24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>11:45</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>ACDR2026 Summary and Closing Remarks</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>所要15分。Summary（宮木所長＝Executive Director）6分＋閉会挨拶 2名×3分（三浦センター長＝Chairman、SCDF 代表【TBC】）＋MC連絡3分。</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="6" t="n"/>
-      <c r="P25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>TS まとめ</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>PPT 19: Wrap-up</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>[Co-Chair, 8 minutes: three to four take-aways across the six presentations; how they answer the session question; items for the conference summary.]
+[Moderator:] Thank you, Dr. Mizan, and thank you to all six presenters. This concludes the Technical Session. Coffee is served in front of the room; please be back by 11:45 for the summary and closing.</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>TS 要旨は原稿ベースで事前に概要案（池田・Mizan→Gerry）。</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Co-Chair → Moderator</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>御礼・連絡</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>PPT 19</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="n"/>
+      <c r="P26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>11:30-11:45</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Coffee Break</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Gerry: Summary スライド最終化（RT Part 2・TS を反映）。前方登壇者席の名札を撤去、閉会用に三浦センター長・SCDF代表の席札。</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6" t="n"/>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="6" t="n"/>
+      <c r="P27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
           <t>11:45</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>ACDR2026 Summary and Closing Remarks</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>所要15分。Summary（宮木所長＝Executive Director）6分＋閉会挨拶 2名×3分（三浦センター長＝Chairman、SCDF 代表【TBC】）＋MC連絡3分。</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+      <c r="M28" s="6" t="n"/>
+      <c r="N28" s="6" t="n"/>
+      <c r="O28" s="6" t="n"/>
+      <c r="P28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>PPT 20: Closing Title → PPT 21: ACDR2026 Summary（Gerry 起草・宮木所長発表）</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Ladies and gentlemen, please be seated. We now come to the summary and closing of ACDR2026. First, I invite Mr MIYAKI Kazuhiro, Executive Director of the Asian Disaster Reduction Center, to present the summary of the conference.
 （Summary 約6分）
 Thank you, Mr Miyaki.</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Summary は Gerry が起草（28日夜〜29日朝）、宮木所長（Executive Director、10月時点の肩書）が発表。</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>宮木所長（演台）</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>紹介</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>PPT 20→21</t>
         </is>
       </c>
-      <c r="K26" s="7" t="inlineStr">
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L26" s="7" t="inlineStr">
+      <c r="L29" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O26" s="7" t="inlineStr">
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="P29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>11:51</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Closing Remarks (1) ADRC</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>PPT 22: Name（三浦センター長 Chairman）</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Now I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, for his closing remarks.
 （閉会挨拶 約3分）
 Thank you very much, Professor Miura.</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>原稿: ACDR2026_Closing_Remarks_MIURA_案0929.docx（約3分）。次回 ACDR は仙台開催、APMCDRR と back-to-back、2027年10月（挨拶内で発表）。</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>Prof. Miura（演台）</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>PPT 22</t>
         </is>
       </c>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="inlineStr">
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="N27" s="7" t="inlineStr">
+      <c r="N30" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="O27" s="7" t="inlineStr">
+      <c r="O30" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P27" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="P30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>11:54</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Closing Remarks (2) SCDF</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>PPT 23: Name（SCDF 代表）</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Finally, on behalf of the co-host, I invite [Mr Alan Chow, Director, Planning &amp; Organisation Department, Singapore Civil Defence Force] for the closing remarks.
 （閉会挨拶 約3分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>Commissioner か Alan Chow 氏か Sylvia に確認【TBC】。</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>SCDF（演台）</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="J31" s="7" t="inlineStr">
         <is>
           <t>PPT 23</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="inlineStr">
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
+      <c r="N31" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="O31" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="P31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>11:57</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>閉会・連絡事項</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>PPT 24: Evaluation（QR）→ PPT 25: Field Trip / Parade info → PPT 26: Thank you</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>This brings ACDR2026 to a close. On behalf of the Asian Disaster Reduction Center and the Singapore Civil Defence Force, thank you all for your participation.
 Before you leave, three announcements. First, please take a moment to complete the evaluation form by scanning the QR code on the screen. Second, lunch is served in Hall 3 from 12:00. Third, for those registered for the field trip to the Civil Defence Academy, the bus departs from the EXPO at 13:00; please gather at [meeting point] by 12:50 after lunch. The SCDF Parade starts at 18:00 in Hall 4, followed by the dinner reception in the Garnet Room. Presentation materials will be posted on the ACDR2026 website. Thank you, and see you tomorrow at the SIDEX-ACDR 2026 Conference in Hall 3.</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>評価フォームは ADRC が用意（Google Form 等、URL/QR を PPT 24 に。担当【TBC】）。フィールドトリップ集合場所【TBC】（田中: 名簿・点呼）。パレード前のホテル着替え・再移動は最終案内に記載。</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>読み上げ</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>PPT 24→26</t>
         </is>
       </c>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="K32" s="7" t="n"/>
+      <c r="L32" s="7" t="inlineStr">
         <is>
           <t>Webinar 終了</t>
         </is>
       </c>
-      <c r="M29" s="7" t="inlineStr">
+      <c r="M32" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
+      <c r="N32" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="inlineStr">
+      <c r="O32" s="7" t="n"/>
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>Webinar終了・録画保存</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="6" t="n">
+    <row r="33">
+      <c r="B33" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>撤収</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>事務局撤収（児玉・藤中）、バイ会談、フィールドトリップ引率（荒木田・吉田・田中）。</t>
         </is>
       </c>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="6" t="n"/>
-      <c r="P30" s="6" t="n"/>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="n"/>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="6" t="n"/>
+      <c r="L33" s="6" t="n"/>
+      <c r="M33" s="6" t="n"/>
+      <c r="N33" s="6" t="n"/>
+      <c r="O33" s="6" t="n"/>
+      <c r="P33" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5367,7 +5375,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Instruction for Speakers – Time Allocation: Maximum 4 minutes (Japan and City of Sendai: 5 minutes; partner organisations: 3 minutes)
+          <t>Instruction for Speakers – Time Allocation: Member countries maximum 5 minutes; adviser countries and partner organisations maximum 3 minutes
 First ring: 1 minute left / Second ring: 30 seconds left / Third ring: end of statement</t>
         </is>
       </c>
@@ -5405,7 +5413,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>アルファベット順。未登録国は削除</t>
+          <t>メンバー国アルファベット順（Japan の次に City of Sendai）。未登録国は削除</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5430,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>ADPC / AHA Centre / ADB / New Zealand NEMA / Google / Online (UNDP, WMO)</t>
+          <t>New Zealand NEMA (adviser) / ADPC / ADB / AHA Centre / Google / Online (UNDP, WMO)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -5432,7 +5440,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>ロゴ使用は各組織の了承要</t>
+          <t>アドバイザー国→ADPC→その他アルファベット順。ロゴ使用は各組織の了承要</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ACDR2026 scenario: set-up from 08:00, one ADRC camera
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -713,7 +713,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -724,7 +724,7 @@
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>会場入室（EXPO確認中）。演台・U字卓上マイク・PC・スクリーン・Zoom・AI通訳・録画のテスト。事務局部屋（Tourmaline 207）立上げ。</t>
+          <t>会場入室（Expo の最早は 08:00 と Sylvia〈JM6〉。07:30 入室は未承認・確認中）。演台・U字卓上マイク・PC・スクリーン・Zoom・AI通訳・録画のテスト。事務局部屋（Tourmaline 207）立上げ。</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
@@ -742,7 +742,7 @@
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>07:30-09:30</t>
+          <t>08:00-09:30</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -759,7 +759,7 @@
         <is>
           <t>- PC（発表用・Zoom用）とスクリーン切替をAVオペと確認
 - 卓上マイク（U字14本＋教室列2本）、スタンド4、ハンド2、演台マイクの音出し
-- Zoom Webinar 起動（神戸: 中村）、カメラ2台の画角（演台／U字パン）確認
+- Zoom Webinar 起動（神戸: 中村）、ADRC 持込カメラ（Zoom 用、HDMI）の画角確認。2台目（U字パン）は未決
 - AI通訳の日本語出力を神戸で確認
 - 名札・国旗プレートを配席表（0928）どおり配置</t>
         </is>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -3316,7 +3316,7 @@
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>TS 用に前方登壇者席（8席）を設置、演台・クリッカー・返しモニター確認。登壇者集合 08:30（池田）、スライド最終確認、Zoom 接続確認（オンライン登壇者があれば 08:45 接続テスト）。</t>
+          <t>入室 08:00（Expo 最早）。RT(2) 09:00 開始まで1時間: TS 用の前方登壇者席（8席）設置、演台・クリッカー・返しモニター確認、登壇者集合 08:30（池田）、スライド最終確認、Zoom 接続確認（オンライン登壇者があれば 08:45 接続テスト）。</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
@@ -3334,7 +3334,7 @@
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>07:30-08:55</t>
+          <t>08:00-08:55</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: Joint Opening programme from Sylvia; ACDR Opening order question
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P40"/>
+  <dimension ref="B1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -814,18 +814,18 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Pre-opening</t>
+          <t>（参考）Joint Opening Ceremony（Hall 3、SIDEX/COSEM 進行）</t>
         </is>
       </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>昼食（Hall 3, 11:45-12:45）から参加者がPeridotへ戻る。VIP（Commissioner、林副大臣、三浦センター長）は12:40までに着席。</t>
+          <t>Sylvia 9/30 共有: 09:00-10:00 登録、10:00-10:05 オープニング映像、10:05-10:15 GOH Ms Sim Ann（Second Minister for Foreign Affairs / Home Affairs）、10:15-10:20 内閣府 林副大臣（5分、NFEC より先＝protocol 上位）、10:20-10:30 NFEC Chairman Mr Markham Shaw、10:30-11:15 FiSAC Keynote 1（Prof Guillermo Rein, Imperial College）、11:15-11:45 SCDF Sharing（SAC Ryan Ong）。ADRC 参加者の 10:30 以降の動線は協議中（FiSAC 出席は協定外、展示会見学を主張）。</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -843,58 +843,42 @@
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>12:30-12:44</t>
+          <t>10:30-11:45</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>参加者誘導・着席</t>
+          <t>ADRC 参加者の動線【協議中】</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>PPT 01: Main Title「ACDR2026 will begin shortly」</t>
+          <t>―</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>（MC 12:40）Ladies and gentlemen, the Asian Conference on Disaster Reduction 2026 will begin shortly. Please take your seats. Delegates of ADRC member countries, please be seated at the U-shaped table where your country name plate is placed.</t>
+          <t>案（ADRC）: GOH 一行が Hall 3 を出た後、ADRC 職員が GOH ルートを避けて展示会へ誘導、日本パビリオンは GOH 通過後に訪問。11:45 昼食（Hall 3）。</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>受付（藤中・田中）でIDストラップ確認。U字＝国名プレート席、2列目＝国名プレート、教室列＝指定席（PNG/PK/ROK/AHA/ADPC/Google/ADB/仙台）、他は自由席。</t>
+          <t>Sylvia 折衷案（FiSAC 基調講演出席→11:15 自由見学）は協定第10条の Event 構成に含まれないため未了解。Commissioner の再承認待ち。</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>会場</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>読み上げ</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>PPT 01</t>
-        </is>
-      </c>
+          <t>ADRC 職員（宮木・児玉・荒木田は VIP 随行）</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>Webinar 参加者入室開始</t>
-        </is>
-      </c>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="7" t="n"/>
       <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="inlineStr">
-        <is>
-          <t>Webinar開始・録画開始</t>
-        </is>
-      </c>
+      <c r="P7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="6" t="n">
@@ -902,18 +886,18 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>ACDR2026 Opening</t>
+          <t>Pre-opening</t>
         </is>
       </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>所要15分。挨拶3名×4分＋MC。写真撮影は大使公邸レセプション（27日）で実施済み。会場バナー前の撮影は Sylvia が配置を検討中【TBC】。</t>
+          <t>昼食（Hall 3, 11:45-12:45）から参加者がPeridotへ戻る。VIP（Commissioner、林副大臣、三浦センター長）は12:40までに着席。</t>
         </is>
       </c>
       <c r="G8" s="6" t="n"/>
@@ -931,2243 +915,2331 @@
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="inlineStr">
         <is>
+          <t>12:30-12:44</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>参加者誘導・着席</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>PPT 01: Main Title「ACDR2026 will begin shortly」</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>（MC 12:40）Ladies and gentlemen, the Asian Conference on Disaster Reduction 2026 will begin shortly. Please take your seats. Delegates of ADRC member countries, please be seated at the U-shaped table where your country name plate is placed.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>受付（藤中・田中）でIDストラップ確認。U字＝国名プレート席、2列目＝国名プレート、教室列＝指定席（PNG/PK/ROK/AHA/ADPC/Google/ADB/仙台）、他は自由席。</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>会場</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>読み上げ</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>PPT 01</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Webinar 参加者入室開始</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Webinar開始・録画開始</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>ACDR2026 Opening</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>所要15分。挨拶3名×4分＋MC。写真撮影は大使公邸レセプション（27日）で実施済み。会場バナー前の撮影は Sylvia が配置を検討中【TBC】。</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>開会・注意事項</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>PPT 02: ACDR2026 Title</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Good afternoon, Excellencies, distinguished delegates, ladies and gentlemen. Welcome to the Asian Conference on Disaster Reduction 2026, ACDR2026, held jointly with SIDEX 2026 and co-hosted by the Asian Disaster Reduction Center and the Singapore Civil Defence Force. I am Lieutenant Colonel Chen Yong Kai of the Singapore Civil Defence Force, and I will be your emcee for the ACDR sessions.
 A few housekeeping notes before we begin. First, this conference is conducted in English. Second, the sessions are being recorded and streamed online to registered participants. Third, for the Roundtable this afternoon, each delegation will make a statement from its seat using the table microphone. Please keep to the time allocation. Finally, please switch your mobile phones to silent mode.</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>日本語AI通訳は Zoom 内のみ（会場では案内しない）。Q&amp;A の方式（RT はコメント用紙／Web フォーム）は 9/30 までに決定【TBC】。</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>日本語AI通訳は Zoom 内のみ（会場では案内しない）。Q&amp;A の方式は吉田・Gerry 回答待ち（10/3）。登壇順は 0925 アジェンダどおり Commissioner→林副大臣→三浦センター長で各4分（Sylvia 9/30「Chairman→Comr か、Comr の持ち時間は」と照会中。3名で15分のため各4分＋MC）。</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>MC at lectern</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>読み上げ</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>PPT 02</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>記録開始</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>記録開始</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="O11" s="7" t="inlineStr">
         <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="P9" s="7" t="inlineStr">
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>12:47</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Opening Remarks (1) SCDF</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>PPT 03: Opening Remarks（3名の氏名・肩書）→ PPT 04: Name（Commissioner）</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>It is now my honour to invite Commissioner Eric Yap Wee Teck, Commissioner of the Singapore Civil Defence Force, to deliver his opening remarks. Commissioner, please.
 （挨拶 約4分）
 Thank you very much, Commissioner Yap.</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Commissioner 出席は【TBC】（原稿は COSEM 側が起案し日本側と共有）。不在時は Mr Alan Chow, Director, Planning &amp; Organisation Department, SCDF。</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Commissioner Yap（演台）</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>PPT 03→04</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="N12" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="O10" s="7" t="inlineStr">
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P10" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="P12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>12:51</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Opening Remarks (2) Government of Japan</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>PPT 05: Name（林副大臣）</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Next, I am pleased to invite Mr HAYASHI Masamichi, Deputy Minister, Government of Japan, to deliver his opening remarks. Deputy Minister Hayashi, please.
 （挨拶 約4分）
 Thank you very much, Deputy Minister Hayashi.</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>逐次通訳を入れると所要が倍になる。日本語で話す場合は英訳原稿を事前配布し通訳は要点のみ、または英語原稿の読み上げ。使用言語・通訳の方式は内閣府に確認【TBC・ADRC→内閣府】。挨拶後、林副大臣は Japan 席に着席、その後退席（Japan 席は内閣府参事官に交代）。</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Deputy Minister（演台）＋通訳</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>PPT 05</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>演台マイク（通訳用ハンド1）</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N13" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr">
+      <c r="O13" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="P13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Opening Remarks (3) ADRC</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>PPT 06: Name（三浦センター長）</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Lastly, I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, to welcome you to the conference. Professor Miura, please.
 （挨拶 約4分：別紙 Opening Remarks 案）
 Thank you very much, Professor Miura.</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>原稿: ACDR2026_Opening_Remarks_MIURA_案0929.docx（英語読み上げ、4分＝約480語）。</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Prof. Miura（演台）</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>PPT 06</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>演台マイク</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>カメラ: 演台</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="N14" s="7" t="inlineStr">
         <is>
           <t>要旨</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="O14" s="7" t="inlineStr">
         <is>
           <t>登壇写真</t>
         </is>
       </c>
-      <c r="P12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>12:59</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Opening → RT へ引継ぎ</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>PPT 07: Roundtable Title</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thank you to all three speakers. This concludes the opening of ACDR2026. We will now proceed directly to the Roundtable Session, Part 1. </t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>会場バナー前で集合写真を撮る場合はここに3分追加（Sylvia 検討中）→ RT 開始 13:03。</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>読み上げ</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>PPT 07</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>（集合写真）</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Roundtable Session Part 1: Progress and Remaining Challenges in Implementing SFDRR 2015-2030</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Moderator: SCDF（LTC Chen Yong Kai）。Co-Moderator: ADRC メンバー国【TBC】。ADRC 運営: 吉田（PIC・進行補助・ベル）、Gerry（ノート・サマリー）、池田（PC・スクリーン）、荒木田（AV/Zoom）。</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="6" t="n"/>
-      <c r="P14" s="6" t="n"/>
+      <c r="P14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Opening → RT へ引継ぎ</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>PPT 07: Roundtable Title</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thank you to all three speakers. This concludes the opening of ACDR2026. We will now proceed directly to the Roundtable Session, Part 1. </t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>会場バナー前で集合写真を撮る場合はここに3分追加（Sylvia 検討中）→ RT 開始 13:03。</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>読み上げ</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>PPT 07</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="n"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>（集合写真）</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Roundtable Session Part 1: Progress and Remaining Challenges in Implementing SFDRR 2015-2030</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Moderator: SCDF（LTC Chen Yong Kai）。Co-Moderator: ADRC メンバー国【TBC】。ADRC 運営: 吉田（PIC・進行補助・ベル）、Gerry（ノート・サマリー）、池田（PC・スクリーン）、荒木田（AV/Zoom）。</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>RT 趣旨説明・進め方</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>PPT 07: RT Title（Moderator / Co-Moderator）→ PPT 08: Instruction for Speakers（時間・ベル）</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Excellencies, distinguished delegates. The Roundtable is the session where ADRC member countries and partners share, in their own words, the progress they have made under the Sendai Framework for Disaster Risk Reduction and the challenges that remain as we approach 2030. Part 1 is held this afternoon and Part 2 tomorrow morning at 9 o’clock.
 Member countries are invited to make a statement of up to five minutes, in alphabetical order; adviser countries and partner organisations will follow with up to three minutes each. Please speak from your seat using the table microphone. A bell will ring once when one minute remains, twice at thirty seconds, and three times at the end of your time. To keep the programme on schedule, I ask all speakers to observe the time strictly.
 Questions and comments will not be taken on the floor during the statements; please write them on the comment sheet at your seat [or submit them via the online form shown on the screen]. They will be shared with the speakers and reflected in the conference summary.</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Co-Moderator を置く場合はここで紹介し、後半（国際機関）の進行を任せる案。ベルは吉田。Q&amp;A方式【TBC】。</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Moderator（モデレーター卓）</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>進行</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>PPT 07→08</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>モデレーター卓マイク</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>カメラ: U字パン</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>13:03</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Armenia</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>PPT 09-1: Armenia</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Armenia. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>アルメニアとアゼルバイジャンは配席上離してあるが、発言順はアルファベット順で連続（荒木田 9/29 決定）。</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N16" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P16" s="7" t="inlineStr">
+      <c r="P18" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>13:08</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Azerbaijan</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>PPT 09-2: Azerbaijan</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Azerbaijan. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>13:13</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Bangladesh</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>PPT 09-3: Bangladesh</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Bangladesh. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L20" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P18" s="7" t="inlineStr">
+      <c r="P20" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>13:18</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Bhutan</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>PPT 09-4: Bhutan</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Bhutan. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L21" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr">
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P19" s="7" t="inlineStr">
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>13:23</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Brunei Darussalam</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>PPT 09-5: Brunei Darussalam</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Brunei Darussalam. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="L22" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr">
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P20" s="7" t="inlineStr">
+      <c r="P22" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>13:28</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Cambodia</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>PPT 09-6: Cambodia</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Cambodia. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L23" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P21" s="7" t="inlineStr">
+      <c r="P23" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>13:33</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Fiji</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>PPT 09-7: Fiji</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Fiji. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L22" s="7" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O22" s="7" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P22" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>13:38</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of India</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>PPT 09-8: India</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of India. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L23" s="7" t="inlineStr">
+      <c r="L25" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P23" s="7" t="inlineStr">
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>13:43</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Japan</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>PPT 09-9: Japan</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Japan, Cabinet Office. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>林副大臣は Opening 後に退席予定のため、日本のステートメントは内閣府参事官【TBC】。</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K24" s="7" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L24" s="7" t="inlineStr">
+      <c r="L26" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M24" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N24" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O24" s="7" t="inlineStr">
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P24" s="7" t="inlineStr">
+      <c r="P26" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>13:48</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Statement: Mr TAKAHASHI Shinichi</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>PPT 09-10: City of Sendai</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite Mr TAKAHASHI Shinichi, Vice Mayor of the City of Sendai, Japan. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>日本の直後に仙台市（教室列1列目の卓上マイク）。次期 APMCDRR・ACDR2027 ホスト市としての紹介を含む見込み。</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K25" s="7" t="inlineStr">
+      <c r="K27" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L25" s="7" t="inlineStr">
+      <c r="L27" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M25" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N25" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O25" s="7" t="inlineStr">
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P25" s="7" t="inlineStr">
+      <c r="P27" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>13:53</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Lao PDR</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>PPT 09-11: Lao PDR</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Lao PDR. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K26" s="7" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L26" s="7" t="inlineStr">
+      <c r="L28" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O26" s="7" t="inlineStr">
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P26" s="7" t="inlineStr">
+      <c r="P28" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>13:58</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Malaysia</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>PPT 09-12: Malaysia</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Malaysia. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L27" s="7" t="inlineStr">
+      <c r="L29" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M27" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N27" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr">
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P27" s="7" t="inlineStr">
+      <c r="P29" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>14:03</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Maldives</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>PPT 09-13: Maldives</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Maldives. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L28" s="7" t="inlineStr">
+      <c r="L30" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M28" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N28" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O30" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P28" s="7" t="inlineStr">
+      <c r="P30" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>14:08</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Mongolia</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>PPT 09-14: Mongolia</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Mongolia. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="J31" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="L31" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M29" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N29" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O29" s="7" t="inlineStr">
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P29" s="7" t="inlineStr">
+      <c r="P31" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>14:13</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Myanmar</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>PPT 09-15: Myanmar</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Myanmar. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K30" s="7" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L30" s="7" t="inlineStr">
+      <c r="L32" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M30" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N30" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O30" s="7" t="inlineStr">
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O32" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P30" s="7" t="inlineStr">
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>14:18</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Pakistan</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>PPT 09-16: Pakistan</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Pakistan. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K31" s="7" t="inlineStr">
+      <c r="K33" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L31" s="7" t="inlineStr">
+      <c r="L33" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M31" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="inlineStr">
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P31" s="7" t="inlineStr">
+      <c r="P33" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>14:23</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Papua New Guinea</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>PPT 09-17: Papua New Guinea</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Papua New Guinea. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K32" s="7" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L32" s="7" t="inlineStr">
+      <c r="L34" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M32" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O32" s="7" t="inlineStr">
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O34" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P32" s="7" t="inlineStr">
+      <c r="P34" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Republic of Korea</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>PPT 09-18: Republic of Korea</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Republic of Korea. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K33" s="7" t="inlineStr">
+      <c r="K35" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L33" s="7" t="inlineStr">
+      <c r="L35" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M33" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N33" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O33" s="7" t="inlineStr">
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P33" s="7" t="inlineStr">
+      <c r="P35" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>14:33</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Singapore</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>PPT 09-19: Singapore</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Singapore. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>アルファベット順どおり Singapore の位置。Commissioner か Alan Chow 氏か【TBC】。</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H36" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr">
+      <c r="K36" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L34" s="7" t="inlineStr">
+      <c r="L36" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N34" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O34" s="7" t="inlineStr">
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O36" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P34" s="7" t="inlineStr">
+      <c r="P36" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>14:38</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Sri Lanka</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>PPT 09-20: Sri Lanka</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Sri Lanka. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K35" s="7" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L35" s="7" t="inlineStr">
+      <c r="L37" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M35" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N35" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O35" s="7" t="inlineStr">
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P35" s="7" t="inlineStr">
+      <c r="P37" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>14:43</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Thailand</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>PPT 09-21: Thailand</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Thailand. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H38" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K36" s="7" t="inlineStr">
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L36" s="7" t="inlineStr">
+      <c r="L38" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M36" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N36" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O36" s="7" t="inlineStr">
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O38" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P36" s="7" t="inlineStr">
+      <c r="P38" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>14:48</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>Statement: the delegation of Turkiye</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>PPT 09-22: Turkiye</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Next, I would like to invite the delegation of Turkiye. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>登録状況（9/16版リスト＋追加）で最終確認。未登録国は行を削除。</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>着席発言（卓上マイク）</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>紹介・御礼</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>国名スライド</t>
         </is>
       </c>
-      <c r="K37" s="7" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>卓上マイク ON 確認</t>
         </is>
       </c>
-      <c r="L37" s="7" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>カメラ: 発言者</t>
         </is>
       </c>
-      <c r="M37" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N37" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O37" s="7" t="inlineStr">
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr">
         <is>
           <t>発言者写真</t>
         </is>
       </c>
-      <c r="P37" s="7" t="inlineStr">
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>Q&amp;A欄監視</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>14:53</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>予備時間・Part 1 締め</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>PPT 11: Comments &amp; Questions（提出方法）</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>We have a few minutes before the end of Part 1. If any delegation wishes to add a brief comment on what we have heard, please raise your name plate. [If none:] Please also use the comment sheets on your desk; they will be collected by the secretariat during the coffee break.</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>進行が押した場合はこの枠を吸収に使う。</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>Moderator</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I40" s="7" t="inlineStr">
         <is>
           <t>進行</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="J40" s="7" t="inlineStr">
         <is>
           <t>PPT 11</t>
         </is>
       </c>
-      <c r="K38" s="7" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
         <is>
           <t>スタンド/ハンドマイク</t>
         </is>
       </c>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="N38" s="7" t="inlineStr">
-        <is>
-          <t>記録</t>
-        </is>
-      </c>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="L40" s="7" t="n"/>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="O40" s="7" t="n"/>
+      <c r="P40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>14:55</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>RT Part 1 まとめ・連絡事項</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>PPT 12: Info（Coffee / SC / Gala）</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>Thank you to all the delegations for your statements. This concludes Part 1 of the Roundtable. The remaining statements will be heard tomorrow morning in Part 2, starting at 9 o’clock sharp in this room.
 Three announcements. First, coffee is served in front of this room. Second, the Steering Committee Meeting for ADRC member countries only will start at 15:15 in this room. Delegates of member countries, please return by 15:15. Third, for participants attending the SIDEX Gala Dinner, the bus leaves Dorsett Changi City Hotel at 17:30. Thank you.</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>SC の前方席: 議長＝内閣府参事官、ADRC（所長）。SC 開始までに机上の RT 資料を回収（吉田・塩見）。</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>Moderator</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>読み上げ</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>PPT 12</t>
         </is>
       </c>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="inlineStr">
+      <c r="K41" s="7" t="n"/>
+      <c r="L41" s="7" t="inlineStr">
         <is>
           <t>Webinar 一時停止（SC は別 Zoom）</t>
         </is>
       </c>
-      <c r="M39" s="7" t="inlineStr">
+      <c r="M41" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="N39" s="7" t="inlineStr">
+      <c r="N41" s="7" t="inlineStr">
         <is>
           <t>記録終了</t>
         </is>
       </c>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="7" t="inlineStr">
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="7" t="inlineStr">
         <is>
           <t>録画停止・保存</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>15:00-15:15</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Coffee Break</t>
         </is>
       </c>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>コーヒー: Peridot 前。SC 用に前方席の名札を差し替え（吉田・田中）。Gerry は RT ノートを整理し Summary 執筆へ。</t>
         </is>
       </c>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
-      <c r="M40" s="6" t="n"/>
-      <c r="N40" s="6" t="n"/>
-      <c r="O40" s="6" t="n"/>
-      <c r="P40" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="6" t="n"/>
+      <c r="K42" s="6" t="n"/>
+      <c r="L42" s="6" t="n"/>
+      <c r="M42" s="6" t="n"/>
+      <c r="N42" s="6" t="n"/>
+      <c r="O42" s="6" t="n"/>
+      <c r="P42" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ACDR2026: opening order per SCDF preference (Chairman, Commissioner, Deputy Minister, tbc)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案0929.xlsx
@@ -1024,7 +1024,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>日本語AI通訳は Zoom 内のみ（会場では案内しない）。Q&amp;A の方式は吉田・Gerry 回答待ち（10/3）。登壇順は 0925 アジェンダどおり Commissioner→林副大臣→三浦センター長で各4分（Sylvia 9/30「Chairman→Comr か、Comr の持ち時間は」と照会中。3名で15分のため各4分＋MC）。</t>
+          <t>日本語AI通訳は Zoom 内のみ（会場では案内しない）。Q&amp;A の方式は吉田・Gerry 回答待ち（10/3）。登壇順はシンガポール側の意向を尊重（荒木田 9/30）: 暫定で三浦センター長→Commissioner→林副大臣（後の登壇者ほど上位とするプロトコル）。SCDF の確認で確定。各4分＋MC 3分。</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1078,29 +1078,29 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Opening Remarks (1) SCDF</t>
+          <t>Opening Remarks (1) ADRC</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>PPT 03: Opening Remarks（3名の氏名・肩書）→ PPT 04: Name（Commissioner）</t>
+          <t>PPT 03: Opening Remarks（3名の氏名・肩書）→ PPT 04: Name（三浦センター長）</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>It is now my honour to invite Commissioner Eric Yap Wee Teck, Commissioner of the Singapore Civil Defence Force, to deliver his opening remarks. Commissioner, please.
-（挨拶 約4分）
-Thank you very much, Commissioner Yap.</t>
+          <t>First, I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, to welcome you to the conference. Professor Miura, please.
+（挨拶 約4分：別紙 Opening Remarks 案）
+Thank you very much, Professor Miura.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Commissioner 出席は【TBC】（原稿は COSEM 側が起案し日本側と共有）。不在時は Mr Alan Chow, Director, Planning &amp; Organisation Department, SCDF。</t>
+          <t>原稿: ACDR2026_Opening_Remarks_MIURA_案0929.docx（英語読み上げ、4分＝約480語）。</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Commissioner Yap（演台）</t>
+          <t>Prof. Miura（演台）</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -1149,29 +1149,29 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Opening Remarks (2) Government of Japan</t>
+          <t>Opening Remarks (2) SCDF</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>PPT 05: Name（林副大臣）</t>
+          <t>PPT 05: Name（Commissioner）</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Next, I am pleased to invite Mr HAYASHI Masamichi, Deputy Minister, Government of Japan, to deliver his opening remarks. Deputy Minister Hayashi, please.
+          <t>Next, it is my honour to invite Commissioner Eric Yap Wee Teck, Commissioner of the Singapore Civil Defence Force, to deliver his opening remarks. Commissioner, please.
 （挨拶 約4分）
-Thank you very much, Deputy Minister Hayashi.</t>
+Thank you very much, Commissioner Yap.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>逐次通訳を入れると所要が倍になる。日本語で話す場合は英訳原稿を事前配布し通訳は要点のみ、または英語原稿の読み上げ。使用言語・通訳の方式は内閣府に確認【TBC・ADRC→内閣府】。挨拶後、林副大臣は Japan 席に着席、その後退席（Japan 席は内閣府参事官に交代）。</t>
+          <t>Commissioner 出席は【TBC】（原稿は COSEM 側が起案し日本側と共有）。不在時は Mr Alan Chow, Director, Planning &amp; Organisation Department, SCDF。</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Deputy Minister（演台）＋通訳</t>
+          <t>Commissioner Yap（演台）</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>演台マイク（通訳用ハンド1）</t>
+          <t>演台マイク</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -1220,29 +1220,29 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Opening Remarks (3) ADRC</t>
+          <t>Opening Remarks (3) Government of Japan</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>PPT 06: Name（三浦センター長）</t>
+          <t>PPT 06: Name（林副大臣）</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Lastly, I would like to invite Professor MIURA Fusanori, Chairman of the Asian Disaster Reduction Center, to welcome you to the conference. Professor Miura, please.
-（挨拶 約4分：別紙 Opening Remarks 案）
-Thank you very much, Professor Miura.</t>
+          <t>Lastly, I am pleased to invite Mr HAYASHI Masamichi, Deputy Minister, Government of Japan, to deliver his opening remarks. Deputy Minister Hayashi, please.
+（挨拶 約4分）
+Thank you very much, Deputy Minister Hayashi.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>原稿: ACDR2026_Opening_Remarks_MIURA_案0929.docx（英語読み上げ、4分＝約480語）。</t>
+          <t>逐次通訳を入れると所要が倍になる。日本語で話す場合は英訳原稿を事前配布し通訳は要点のみ、または英語原稿の読み上げ。使用言語・通訳の方式は内閣府に確認【TBC・ADRC→内閣府】。挨拶後、林副大臣は Japan 席に着席、その後退席（Japan 席は内閣府参事官に交代）。</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Prof. Miura（演台）</t>
+          <t>Deputy Minister（演台）＋通訳</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>演台マイク</t>
+          <t>演台マイク（通訳用ハンド1）</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
@@ -5363,10 +5363,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Opening Remarks:
+          <t>Opening Remarks (order per SCDF, tbc):
+– Prof. MIURA Fusanori, Chairman, Asian Disaster Reduction Center
 – Mr Eric Yap Wee Teck, Commissioner, Singapore Civil Defence Force (tbc)
 – Mr HAYASHI Masamichi, Deputy Minister, Government of Japan
-– Prof. MIURA Fusanori, Chairman, Asian Disaster Reduction Center
 Emcee: LTC Chen Yong Kai, SCDF</t>
         </is>
       </c>

</xml_diff>